<commit_message>
Aggiunta campo squadra per sviluppi futuri
</commit_message>
<xml_diff>
--- a/tables/xls/it/60_Volontari.xlsx
+++ b/tables/xls/it/60_Volontari.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="93">
   <si>
     <t>ORGANIZZAZIONE</t>
   </si>
@@ -70,6 +70,9 @@
   </si>
   <si>
     <t>TURNO</t>
+  </si>
+  <si>
+    <t>SQUADRA</t>
   </si>
   <si>
     <t>CODICE BADGE</t>
@@ -631,7 +634,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:Z1"/>
+  <dimension ref="A1:AA1"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="17.567" bestFit="true" customWidth="true" style="0"/>
@@ -652,17 +655,18 @@
     <col min="16" max="16" width="23.423" bestFit="true" customWidth="true" style="0"/>
     <col min="17" max="17" width="25.851" bestFit="true" customWidth="true" style="0"/>
     <col min="18" max="18" width="6.998" bestFit="true" customWidth="true" style="0"/>
-    <col min="19" max="19" width="15.282" bestFit="true" customWidth="true" style="0"/>
-    <col min="20" max="20" width="21.138" bestFit="true" customWidth="true" style="0"/>
-    <col min="21" max="21" width="25.851" bestFit="true" customWidth="true" style="0"/>
-    <col min="22" max="22" width="23.423" bestFit="true" customWidth="true" style="0"/>
-    <col min="23" max="23" width="26.993" bestFit="true" customWidth="true" style="0"/>
-    <col min="24" max="24" width="31.707" bestFit="true" customWidth="true" style="0"/>
-    <col min="25" max="25" width="5.856" bestFit="true" customWidth="true" style="0"/>
-    <col min="26" max="26" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="19" max="19" width="9.283" bestFit="true" customWidth="true" style="0"/>
+    <col min="20" max="20" width="15.282" bestFit="true" customWidth="true" style="0"/>
+    <col min="21" max="21" width="21.138" bestFit="true" customWidth="true" style="0"/>
+    <col min="22" max="22" width="25.851" bestFit="true" customWidth="true" style="0"/>
+    <col min="23" max="23" width="23.423" bestFit="true" customWidth="true" style="0"/>
+    <col min="24" max="24" width="26.993" bestFit="true" customWidth="true" style="0"/>
+    <col min="25" max="25" width="31.707" bestFit="true" customWidth="true" style="0"/>
+    <col min="26" max="26" width="5.856" bestFit="true" customWidth="true" style="0"/>
+    <col min="27" max="27" width="12.854" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26">
+    <row r="1" spans="1:27">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -740,6 +744,9 @@
       </c>
       <c r="Z1" t="s">
         <v>25</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -754,10 +761,10 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:AA25"/>
+  <dimension ref="A1:AB25"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:27">
+    <row r="1" spans="1:28">
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -836,10 +843,13 @@
       <c r="AA1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="2" spans="1:27">
+      <c r="AB1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:28">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -896,33 +906,36 @@
         <v>30</v>
       </c>
       <c r="T2">
+        <v>31</v>
+      </c>
+      <c r="U2">
         <v>32</v>
       </c>
-      <c r="U2">
+      <c r="V2">
         <v>33</v>
       </c>
-      <c r="V2">
+      <c r="W2">
         <v>80</v>
       </c>
-      <c r="W2">
+      <c r="X2">
         <v>81</v>
       </c>
-      <c r="X2">
+      <c r="Y2">
         <v>90</v>
       </c>
-      <c r="Y2">
+      <c r="Z2">
         <v>93</v>
       </c>
-      <c r="Z2">
+      <c r="AA2">
         <v>99</v>
       </c>
-      <c r="AA2">
+      <c r="AB2">
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:27">
+    <row r="3" spans="1:28">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B3" t="s">
         <v>0</v>
@@ -949,7 +962,7 @@
         <v>7</v>
       </c>
       <c r="J3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K3" t="s">
         <v>9</v>
@@ -964,7 +977,7 @@
         <v>12</v>
       </c>
       <c r="O3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="P3" t="s">
         <v>14</v>
@@ -973,7 +986,7 @@
         <v>15</v>
       </c>
       <c r="R3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="S3" t="s">
         <v>17</v>
@@ -982,139 +995,145 @@
         <v>18</v>
       </c>
       <c r="U3" t="s">
-        <v>73</v>
+        <v>19</v>
       </c>
       <c r="V3" t="s">
         <v>74</v>
       </c>
       <c r="W3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="X3" t="s">
         <v>77</v>
       </c>
       <c r="Y3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="Z3" t="s">
-        <v>24</v>
+        <v>81</v>
       </c>
       <c r="AA3" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="4" spans="1:27">
+      <c r="AB3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28">
       <c r="A4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="H4" t="s">
+        <v>58</v>
+      </c>
+      <c r="I4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J4" t="s">
+        <v>58</v>
+      </c>
+      <c r="K4" t="s">
+        <v>51</v>
+      </c>
+      <c r="L4" t="s">
+        <v>58</v>
+      </c>
+      <c r="M4" t="s">
+        <v>58</v>
+      </c>
+      <c r="N4" t="s">
+        <v>58</v>
+      </c>
+      <c r="O4" t="s">
+        <v>58</v>
+      </c>
+      <c r="P4" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>70</v>
+      </c>
+      <c r="R4" t="s">
+        <v>51</v>
+      </c>
+      <c r="S4" t="s">
+        <v>51</v>
+      </c>
+      <c r="T4" t="s">
+        <v>51</v>
+      </c>
+      <c r="U4" t="s">
+        <v>51</v>
+      </c>
+      <c r="V4" t="s">
+        <v>51</v>
+      </c>
+      <c r="W4" t="s">
         <v>57</v>
       </c>
-      <c r="I4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J4" t="s">
+      <c r="X4" t="s">
         <v>57</v>
       </c>
-      <c r="K4" t="s">
-        <v>50</v>
-      </c>
-      <c r="L4" t="s">
-        <v>57</v>
-      </c>
-      <c r="M4" t="s">
-        <v>57</v>
-      </c>
-      <c r="N4" t="s">
-        <v>57</v>
-      </c>
-      <c r="O4" t="s">
-        <v>57</v>
-      </c>
-      <c r="P4" t="s">
-        <v>57</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>69</v>
-      </c>
-      <c r="R4" t="s">
-        <v>50</v>
-      </c>
-      <c r="S4" t="s">
-        <v>50</v>
-      </c>
-      <c r="T4" t="s">
-        <v>50</v>
-      </c>
-      <c r="U4" t="s">
-        <v>50</v>
-      </c>
-      <c r="V4" t="s">
-        <v>56</v>
-      </c>
-      <c r="W4" t="s">
-        <v>56</v>
-      </c>
-      <c r="X4" t="s">
-        <v>78</v>
-      </c>
       <c r="Y4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Z4" t="s">
-        <v>50</v>
+        <v>79</v>
       </c>
       <c r="AA4" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="5" spans="1:27">
+        <v>51</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28">
       <c r="A5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="J5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="L5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="P5" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="6" spans="1:27">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28">
       <c r="A6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B6">
         <v>255</v>
@@ -1194,476 +1213,491 @@
       <c r="AA6">
         <v>255</v>
       </c>
-    </row>
-    <row r="7" spans="1:27">
+      <c r="AB6">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28">
       <c r="A7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="I7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="L7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="M7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="O7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="P7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="R7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="S7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="T7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="U7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="V7" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="W7" t="s">
         <v>52</v>
       </c>
       <c r="X7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Y7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Z7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="AA7" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="8" spans="1:27">
+        <v>53</v>
+      </c>
+      <c r="AB7" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28">
       <c r="A8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I8" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="J8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="P8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S8" t="s">
-        <v>71</v>
-      </c>
-      <c r="T8" t="s">
         <v>72</v>
       </c>
-      <c r="V8" t="s">
-        <v>75</v>
-      </c>
-      <c r="X8" t="s">
-        <v>79</v>
-      </c>
-      <c r="AA8" t="s">
+      <c r="U8" t="s">
+        <v>73</v>
+      </c>
+      <c r="W8" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>80</v>
+      </c>
+      <c r="AB8" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28">
+      <c r="A9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" t="s">
+        <v>53</v>
+      </c>
+      <c r="C9" t="s">
+        <v>53</v>
+      </c>
+      <c r="D9" t="s">
+        <v>53</v>
+      </c>
+      <c r="E9" t="s">
+        <v>53</v>
+      </c>
+      <c r="F9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G9" t="s">
+        <v>53</v>
+      </c>
+      <c r="H9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I9" t="s">
+        <v>53</v>
+      </c>
+      <c r="J9" t="s">
+        <v>53</v>
+      </c>
+      <c r="K9" t="s">
+        <v>53</v>
+      </c>
+      <c r="L9" t="s">
+        <v>53</v>
+      </c>
+      <c r="M9" t="s">
+        <v>53</v>
+      </c>
+      <c r="N9" t="s">
+        <v>53</v>
+      </c>
+      <c r="O9" t="s">
+        <v>53</v>
+      </c>
+      <c r="P9" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>53</v>
+      </c>
+      <c r="R9" t="s">
+        <v>53</v>
+      </c>
+      <c r="S9" t="s">
+        <v>53</v>
+      </c>
+      <c r="T9" t="s">
+        <v>53</v>
+      </c>
+      <c r="U9" t="s">
+        <v>53</v>
+      </c>
+      <c r="V9" t="s">
+        <v>53</v>
+      </c>
+      <c r="W9" t="s">
+        <v>53</v>
+      </c>
+      <c r="X9" t="s">
+        <v>53</v>
+      </c>
+      <c r="Y9" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>53</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB9" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28">
+      <c r="A10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" t="s">
+        <v>52</v>
+      </c>
+      <c r="C10" t="s">
+        <v>52</v>
+      </c>
+      <c r="D10" t="s">
+        <v>52</v>
+      </c>
+      <c r="E10" t="s">
+        <v>52</v>
+      </c>
+      <c r="F10" t="s">
+        <v>52</v>
+      </c>
+      <c r="G10" t="s">
+        <v>52</v>
+      </c>
+      <c r="H10" t="s">
+        <v>52</v>
+      </c>
+      <c r="I10" t="s">
+        <v>52</v>
+      </c>
+      <c r="J10" t="s">
+        <v>52</v>
+      </c>
+      <c r="K10" t="s">
+        <v>52</v>
+      </c>
+      <c r="L10" t="s">
+        <v>52</v>
+      </c>
+      <c r="M10" t="s">
+        <v>52</v>
+      </c>
+      <c r="N10" t="s">
+        <v>52</v>
+      </c>
+      <c r="O10" t="s">
+        <v>52</v>
+      </c>
+      <c r="P10" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>52</v>
+      </c>
+      <c r="R10" t="s">
+        <v>52</v>
+      </c>
+      <c r="S10" t="s">
+        <v>52</v>
+      </c>
+      <c r="T10" t="s">
+        <v>52</v>
+      </c>
+      <c r="U10" t="s">
+        <v>52</v>
+      </c>
+      <c r="V10" t="s">
+        <v>52</v>
+      </c>
+      <c r="W10" t="s">
+        <v>52</v>
+      </c>
+      <c r="X10" t="s">
+        <v>52</v>
+      </c>
+      <c r="Y10" t="s">
+        <v>52</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>52</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>52</v>
+      </c>
+      <c r="AB10" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28">
+      <c r="A11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" t="s">
+        <v>54</v>
+      </c>
+      <c r="C11" t="s">
+        <v>53</v>
+      </c>
+      <c r="D11" t="s">
+        <v>54</v>
+      </c>
+      <c r="E11" t="s">
+        <v>54</v>
+      </c>
+      <c r="F11" t="s">
+        <v>54</v>
+      </c>
+      <c r="H11" t="s">
+        <v>53</v>
+      </c>
+      <c r="J11" t="s">
+        <v>53</v>
+      </c>
+      <c r="K11" t="s">
+        <v>53</v>
+      </c>
+      <c r="L11" t="s">
+        <v>53</v>
+      </c>
+      <c r="P11" t="s">
+        <v>53</v>
+      </c>
+      <c r="S11" t="s">
+        <v>53</v>
+      </c>
+      <c r="U11" t="s">
+        <v>53</v>
+      </c>
+      <c r="V11" t="s">
+        <v>53</v>
+      </c>
+      <c r="W11" t="s">
+        <v>53</v>
+      </c>
+      <c r="X11" t="s">
+        <v>53</v>
+      </c>
+      <c r="Y11" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>53</v>
+      </c>
+      <c r="AA11" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28">
+      <c r="A12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" t="s">
+        <v>53</v>
+      </c>
+      <c r="C12" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12" t="s">
+        <v>53</v>
+      </c>
+      <c r="E12" t="s">
+        <v>53</v>
+      </c>
+      <c r="F12" t="s">
+        <v>53</v>
+      </c>
+      <c r="G12" t="s">
+        <v>53</v>
+      </c>
+      <c r="H12" t="s">
+        <v>53</v>
+      </c>
+      <c r="I12" t="s">
+        <v>53</v>
+      </c>
+      <c r="J12" t="s">
+        <v>53</v>
+      </c>
+      <c r="K12" t="s">
+        <v>53</v>
+      </c>
+      <c r="L12" t="s">
+        <v>53</v>
+      </c>
+      <c r="M12" t="s">
+        <v>53</v>
+      </c>
+      <c r="N12" t="s">
+        <v>53</v>
+      </c>
+      <c r="O12" t="s">
+        <v>53</v>
+      </c>
+      <c r="P12" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>53</v>
+      </c>
+      <c r="R12" t="s">
+        <v>53</v>
+      </c>
+      <c r="S12" t="s">
+        <v>53</v>
+      </c>
+      <c r="T12" t="s">
+        <v>53</v>
+      </c>
+      <c r="U12" t="s">
+        <v>53</v>
+      </c>
+      <c r="V12" t="s">
+        <v>53</v>
+      </c>
+      <c r="W12" t="s">
+        <v>53</v>
+      </c>
+      <c r="X12" t="s">
+        <v>53</v>
+      </c>
+      <c r="Y12" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>53</v>
+      </c>
+      <c r="AA12" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB12" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="13" spans="1:28">
+      <c r="A13" t="s">
+        <v>38</v>
+      </c>
+      <c r="F13" t="s">
+        <v>56</v>
+      </c>
+      <c r="Z13" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:27">
-      <c r="A9" t="s">
-        <v>33</v>
-      </c>
-      <c r="B9" t="s">
-        <v>52</v>
-      </c>
-      <c r="C9" t="s">
-        <v>52</v>
-      </c>
-      <c r="D9" t="s">
-        <v>52</v>
-      </c>
-      <c r="E9" t="s">
-        <v>52</v>
-      </c>
-      <c r="F9" t="s">
-        <v>52</v>
-      </c>
-      <c r="G9" t="s">
-        <v>52</v>
-      </c>
-      <c r="H9" t="s">
-        <v>52</v>
-      </c>
-      <c r="I9" t="s">
-        <v>52</v>
-      </c>
-      <c r="J9" t="s">
-        <v>52</v>
-      </c>
-      <c r="K9" t="s">
-        <v>52</v>
-      </c>
-      <c r="L9" t="s">
-        <v>52</v>
-      </c>
-      <c r="M9" t="s">
-        <v>52</v>
-      </c>
-      <c r="N9" t="s">
-        <v>52</v>
-      </c>
-      <c r="O9" t="s">
-        <v>52</v>
-      </c>
-      <c r="P9" t="s">
-        <v>52</v>
-      </c>
-      <c r="Q9" t="s">
-        <v>52</v>
-      </c>
-      <c r="R9" t="s">
-        <v>52</v>
-      </c>
-      <c r="S9" t="s">
-        <v>52</v>
-      </c>
-      <c r="T9" t="s">
-        <v>52</v>
-      </c>
-      <c r="U9" t="s">
-        <v>52</v>
-      </c>
-      <c r="V9" t="s">
-        <v>52</v>
-      </c>
-      <c r="W9" t="s">
-        <v>52</v>
-      </c>
-      <c r="X9" t="s">
-        <v>52</v>
-      </c>
-      <c r="Y9" t="s">
-        <v>52</v>
-      </c>
-      <c r="Z9" t="s">
-        <v>52</v>
-      </c>
-      <c r="AA9" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="10" spans="1:27">
-      <c r="A10" t="s">
-        <v>34</v>
-      </c>
-      <c r="B10" t="s">
-        <v>51</v>
-      </c>
-      <c r="C10" t="s">
-        <v>51</v>
-      </c>
-      <c r="D10" t="s">
-        <v>51</v>
-      </c>
-      <c r="E10" t="s">
-        <v>51</v>
-      </c>
-      <c r="F10" t="s">
-        <v>51</v>
-      </c>
-      <c r="G10" t="s">
-        <v>51</v>
-      </c>
-      <c r="H10" t="s">
-        <v>51</v>
-      </c>
-      <c r="I10" t="s">
-        <v>51</v>
-      </c>
-      <c r="J10" t="s">
-        <v>51</v>
-      </c>
-      <c r="K10" t="s">
-        <v>51</v>
-      </c>
-      <c r="L10" t="s">
-        <v>51</v>
-      </c>
-      <c r="M10" t="s">
-        <v>51</v>
-      </c>
-      <c r="N10" t="s">
-        <v>51</v>
-      </c>
-      <c r="O10" t="s">
-        <v>51</v>
-      </c>
-      <c r="P10" t="s">
-        <v>51</v>
-      </c>
-      <c r="Q10" t="s">
-        <v>51</v>
-      </c>
-      <c r="R10" t="s">
-        <v>51</v>
-      </c>
-      <c r="S10" t="s">
-        <v>51</v>
-      </c>
-      <c r="T10" t="s">
-        <v>51</v>
-      </c>
-      <c r="U10" t="s">
-        <v>51</v>
-      </c>
-      <c r="V10" t="s">
-        <v>51</v>
-      </c>
-      <c r="W10" t="s">
-        <v>51</v>
-      </c>
-      <c r="X10" t="s">
-        <v>51</v>
-      </c>
-      <c r="Y10" t="s">
-        <v>51</v>
-      </c>
-      <c r="Z10" t="s">
-        <v>51</v>
-      </c>
-      <c r="AA10" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="11" spans="1:27">
-      <c r="A11" t="s">
-        <v>35</v>
-      </c>
-      <c r="B11" t="s">
-        <v>53</v>
-      </c>
-      <c r="C11" t="s">
-        <v>52</v>
-      </c>
-      <c r="D11" t="s">
-        <v>53</v>
-      </c>
-      <c r="E11" t="s">
-        <v>53</v>
-      </c>
-      <c r="F11" t="s">
-        <v>53</v>
-      </c>
-      <c r="H11" t="s">
-        <v>52</v>
-      </c>
-      <c r="J11" t="s">
-        <v>52</v>
-      </c>
-      <c r="K11" t="s">
-        <v>52</v>
-      </c>
-      <c r="L11" t="s">
-        <v>52</v>
-      </c>
-      <c r="P11" t="s">
-        <v>52</v>
-      </c>
-      <c r="S11" t="s">
-        <v>52</v>
-      </c>
-      <c r="T11" t="s">
-        <v>52</v>
-      </c>
-      <c r="U11" t="s">
-        <v>52</v>
-      </c>
-      <c r="V11" t="s">
-        <v>52</v>
-      </c>
-      <c r="W11" t="s">
-        <v>52</v>
-      </c>
-      <c r="X11" t="s">
-        <v>52</v>
-      </c>
-      <c r="Y11" t="s">
-        <v>52</v>
-      </c>
-      <c r="Z11" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="12" spans="1:27">
-      <c r="A12" t="s">
-        <v>36</v>
-      </c>
-      <c r="B12" t="s">
-        <v>52</v>
-      </c>
-      <c r="C12" t="s">
-        <v>52</v>
-      </c>
-      <c r="D12" t="s">
-        <v>52</v>
-      </c>
-      <c r="E12" t="s">
-        <v>52</v>
-      </c>
-      <c r="F12" t="s">
-        <v>52</v>
-      </c>
-      <c r="G12" t="s">
-        <v>52</v>
-      </c>
-      <c r="H12" t="s">
-        <v>52</v>
-      </c>
-      <c r="I12" t="s">
-        <v>52</v>
-      </c>
-      <c r="J12" t="s">
-        <v>52</v>
-      </c>
-      <c r="K12" t="s">
-        <v>52</v>
-      </c>
-      <c r="L12" t="s">
-        <v>52</v>
-      </c>
-      <c r="M12" t="s">
-        <v>52</v>
-      </c>
-      <c r="N12" t="s">
-        <v>52</v>
-      </c>
-      <c r="O12" t="s">
-        <v>52</v>
-      </c>
-      <c r="P12" t="s">
-        <v>52</v>
-      </c>
-      <c r="Q12" t="s">
-        <v>52</v>
-      </c>
-      <c r="R12" t="s">
-        <v>52</v>
-      </c>
-      <c r="S12" t="s">
-        <v>52</v>
-      </c>
-      <c r="T12" t="s">
-        <v>52</v>
-      </c>
-      <c r="U12" t="s">
-        <v>52</v>
-      </c>
-      <c r="V12" t="s">
-        <v>52</v>
-      </c>
-      <c r="W12" t="s">
-        <v>52</v>
-      </c>
-      <c r="X12" t="s">
-        <v>52</v>
-      </c>
-      <c r="Y12" t="s">
-        <v>52</v>
-      </c>
-      <c r="Z12" t="s">
-        <v>52</v>
-      </c>
-      <c r="AA12" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="13" spans="1:27">
-      <c r="A13" t="s">
-        <v>37</v>
-      </c>
-      <c r="F13" t="s">
+    <row r="14" spans="1:28">
+      <c r="A14" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" t="s">
         <v>55</v>
       </c>
-      <c r="Y13" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="14" spans="1:27">
-      <c r="A14" t="s">
-        <v>38</v>
-      </c>
-      <c r="B14" t="s">
-        <v>54</v>
-      </c>
       <c r="C14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="K14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="R14" t="s">
-        <v>54</v>
-      </c>
-      <c r="U14" t="s">
-        <v>54</v>
-      </c>
-      <c r="Z14" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="15" spans="1:27">
+        <v>55</v>
+      </c>
+      <c r="V14" t="s">
+        <v>55</v>
+      </c>
+      <c r="AA14" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15" spans="1:28">
       <c r="A15" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B15" t="s">
         <v>0</v>
@@ -1689,112 +1723,112 @@
       <c r="R15" t="s">
         <v>16</v>
       </c>
-      <c r="U15" t="s">
-        <v>19</v>
-      </c>
-      <c r="Z15" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="16" spans="1:27">
+      <c r="V15" t="s">
+        <v>20</v>
+      </c>
+      <c r="AA15" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:28">
       <c r="A16" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="J16" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K16" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="L16" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="P16" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="17" spans="1:27">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="17" spans="1:28">
       <c r="A17" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C17" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="18" spans="1:27">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="18" spans="1:28">
       <c r="A18" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B18" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C18" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D18" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="19" spans="1:27">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="19" spans="1:28">
       <c r="A19" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B19" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C19" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D19" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="20" spans="1:27">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="20" spans="1:28">
       <c r="A20" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B20" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:27">
+    <row r="21" spans="1:28">
       <c r="A21" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B21" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="22" spans="1:27">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="22" spans="1:28">
       <c r="A22" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B22" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="23" spans="1:27">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="23" spans="1:28">
       <c r="A23" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B23" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="24" spans="1:27">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="24" spans="1:28">
       <c r="A24" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B24" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="25" spans="1:27">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="25" spans="1:28">
       <c r="A25" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B25" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>